<commit_message>
Add Snowflake dbt CFPB analytics pipeline
</commit_message>
<xml_diff>
--- a/tableau/CFPB_Tableau_Source.xlsx
+++ b/tableau/CFPB_Tableau_Source.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rd8b6c048598340f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Volume" sheetId="2" r:id="R9e06fb5efc4c4468"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Summary" sheetId="3" r:id="R216153c5505c4d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Summary" sheetId="4" r:id="Readbfb20839a447e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Performance" sheetId="5" r:id="Refd89e4a0e194f58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix" sheetId="6" r:id="R009bf6cf9f3347e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Summary" sheetId="7" r:id="R2646e63077814060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R90af673bdef64b20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Volume" sheetId="2" r:id="R9b80de7d0cc0437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Summary" sheetId="3" r:id="R96491d5d6d884fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issue Summary" sheetId="4" r:id="R2825a44162c74a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Response Performance" sheetId="5" r:id="R48c87967e7244ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Channel Mix" sheetId="6" r:id="Rc3e8c65498e1437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="State Summary" sheetId="7" r:id="Ra5069bf998384274"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,31 +406,39 @@
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="11" t="str">
+      <x:c r="A8" s="9" t="str">
+        <x:v>Data mode</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Legacy local-summary fallback — run the Snowflake/dbt pipeline before final Tableau publication</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="11" t="str">
         <x:v>Use</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="str">
-        <x:v>Connect Tableau to the individual summary sheets; do not publish raw data.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="15" t="str">
+      <x:c r="B9" s="12" t="str">
+        <x:v>Connect Tableau to these aggregate sheets. Tableau Public uses this extract snapshot, not a live Snowflake connection.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="15" t="str">
         <x:v>Important note</x:v>
       </x:c>
-      <x:c r="B10" s="15" t="str">
+      <x:c r="B11" s="15" t="str">
         <x:v>The two credit-reporting product labels are kept separate because source taxonomy labels differ. Do not combine them without a documented mapping.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11"/>
-      <x:c r="B11"/>
-    </x:row>
     <x:row r="12">
-      <x:c r="A12" s="16" t="str">
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="16" t="str">
         <x:v>Dashboard build</x:v>
       </x:c>
-      <x:c r="B12" s="16" t="str">
-        <x:v>Use the Tableau build specification in docs/tableau_build_spec.md.</x:v>
+      <x:c r="B13" s="16" t="str">
+        <x:v>Use the Tableau build specification in docs/tableau_build_spec.md. Keep a single dashboard with documented global filters and actions.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>